<commit_message>
Cập nhật trạng thái làm việc hiện tại - tất cả thay đổi đang có
</commit_message>
<xml_diff>
--- a/product Tester/templates/unit_test_login_register.xlsx
+++ b/product Tester/templates/unit_test_login_register.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="8400"/>
+    <workbookView windowWidth="23040" windowHeight="9120"/>
   </bookViews>
   <sheets>
     <sheet name="Unit Test Cases" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="32">
   <si>
     <t>ID</t>
   </si>
@@ -41,21 +41,23 @@
     <t>Expected Result</t>
   </si>
   <si>
+    <t xml:space="preserve">Prerequisite </t>
+  </si>
+  <si>
     <t>TC-01</t>
   </si>
   <si>
     <t>Đăng nhập thành công (Admin)</t>
   </si>
   <si>
-    <t>1. đi tới "https://mini-unigate.fsoft.com.vn/fkr/auth/login".
+    <t xml:space="preserve">1. đi tới "https://mini-unigate.fsoft.com.vn/fkr/auth/login".
 2. Nhập Username: "Admin".
 3. Nhập Password: "fbgsde45634#$%^".
 4. Nhấn nút "Sign in".
-5. di chuột vào "admin"
-6. nhấn "logout"</t>
-  </si>
-  <si>
-    <t>Người dùng được chuyển về trang Sign to get started</t>
+</t>
+  </si>
+  <si>
+    <t>Người dùng được chuyển về trang My Workspace</t>
   </si>
   <si>
     <t>TC-02</t>
@@ -73,6 +75,9 @@
     <t>Hệ thống không cho phép đăng nhập vì nhập sai tài khoản hoặc mật khẩu</t>
   </si>
   <si>
+    <t>TC1-Failed</t>
+  </si>
+  <si>
     <t>TC-03</t>
   </si>
   <si>
@@ -116,6 +121,25 @@
   </si>
   <si>
     <t>Hệ thống hiển tài khoản bị khóa hoặc bị chặn hoặc tài khoản không đúng.</t>
+  </si>
+  <si>
+    <t>TC-06</t>
+  </si>
+  <si>
+    <t>logout</t>
+  </si>
+  <si>
+    <t>1. di chuyển chuột vào "admin"
+2. chọn "logout"</t>
+  </si>
+  <si>
+    <t>Hệ thống trở về trang "Sign in to get started"</t>
+  </si>
+  <si>
+    <t>TC1-Passed</t>
+  </si>
+  <si>
+    <t>TC-07</t>
   </si>
 </sst>
 </file>
@@ -289,7 +313,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="34">
+  <fills count="35">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -300,6 +324,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FF4F81BD"/>
         <bgColor rgb="FF4F81BD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
@@ -634,7 +664,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -658,16 +688,16 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
@@ -676,95 +706,102 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1112,16 +1149,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:D6"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelRow="5" outlineLevelCol="3"/>
+  <dimension ref="A1:E8"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelRow="7" outlineLevelCol="4"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="2" width="30" customWidth="1"/>
     <col min="3" max="3" width="65.8888888888889" customWidth="1"/>
     <col min="4" max="4" width="56" customWidth="1"/>
+    <col min="5" max="5" width="23.1111111111111" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1134,75 +1172,113 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
     </row>
-    <row r="2" ht="86.4" spans="1:4">
-      <c r="A2" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B2" s="2" t="s">
+    <row r="2" ht="72" spans="1:5">
+      <c r="A2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="C2" s="3" t="s">
         <v>7</v>
       </c>
+      <c r="D2" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="4"/>
     </row>
-    <row r="3" ht="57.6" spans="1:4">
-      <c r="A3" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" s="2" t="s">
+    <row r="3" ht="57.6" spans="1:5">
+      <c r="A3" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="B3" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="C3" s="3" t="s">
         <v>11</v>
       </c>
+      <c r="D3" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>13</v>
+      </c>
     </row>
-    <row r="4" ht="57.6" spans="1:4">
-      <c r="A4" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B4" s="2" t="s">
+    <row r="4" ht="57.6" spans="1:5">
+      <c r="A4" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E4" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>15</v>
-      </c>
     </row>
-    <row r="5" ht="57.6" spans="1:4">
-      <c r="A5" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C5" s="2" t="s">
+    <row r="5" ht="57.6" spans="1:5">
+      <c r="A5" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="B5" s="3" t="s">
         <v>19</v>
       </c>
+      <c r="C5" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>13</v>
+      </c>
     </row>
-    <row r="6" ht="57.6" spans="1:4">
-      <c r="A6" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="C6" s="2" t="s">
+    <row r="6" ht="57.6" spans="1:5">
+      <c r="A6" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="B6" s="3" t="s">
         <v>23</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" ht="28.8" spans="1:5">
+      <c r="A7" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1">
+      <c r="A8" t="s">
+        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>